<commit_message>
Finalisation du mode excel
</commit_message>
<xml_diff>
--- a/excel/headers.xlsx
+++ b/excel/headers.xlsx
@@ -22,10 +22,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">size</t>
+    <t xml:space="preserve">nom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">taille</t>
   </si>
   <si>
     <t xml:space="preserve">img_x</t>
@@ -76,6 +76,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -135,8 +136,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -267,46 +272,46 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>